<commit_message>
Sumar campo "Prompt sugerido para IA" a contenidos + plantilla Excel
Nuevo textarea en el modal de Nuevo contenido, entre Texto en pantalla
y ¿Es contenido para pauta?. Se guarda como promptIA, se detecta en el
diff de importación/reimportación (IMPORT_DIFF_FIELDS) y se agregó la
columna correspondiente a la plantilla descargable (con su explicación
en la hoja de Instrucciones).
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
+++ b/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
@@ -85,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -100,6 +100,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -657,100 +660,107 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>• Prompt sugerido para IA: si esa pieza se va a generar con inteligencia artificial, el prompt sugerido para armarla (opcional).</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>VALORES VÁLIDOS POR COLUMNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
+          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
+          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
+          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
+          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
+          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
+          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
+          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
-    </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-    </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos, asignación a alguien del equipo) se completan después, ya adentro del hub.</t>
         </is>
@@ -767,7 +777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -783,7 +793,7 @@
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
@@ -858,25 +868,30 @@
       </c>
       <c r="N1" s="4" t="inlineStr">
         <is>
+          <t>Prompt sugerido para IA</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
           <t>Pauta</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>Link pieza terminada</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>Link material de referencia</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>Notas internas</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Pilar / fase (referencia interna, NO se sube al hub)</t>
         </is>
@@ -948,19 +963,24 @@
           <t>Este es el texto que va escrito ADENTRO de la imagen o el video (distinto del copy de arriba).</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>Ej: "Foto de producto sobre fondo claro, estilo minimalista, luz natural, sin texto superpuesto"</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Solo orgánico</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" s="5" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr"/>
+      <c r="R2" s="5" t="inlineStr">
         <is>
           <t>Ejemplo de fila — borrala y cargá tus propios contenidos.</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="S2" s="5" t="inlineStr">
         <is>
           <t>Septiembre · Ejemplo</t>
         </is>

</xml_diff>

<commit_message>
Sumar campo "Sugerencia de pieza creativa" (visual/secuencia), separado del prompt de IA
Nuevo textarea en Nuevo contenido para describir la pieza visualmente
-- descripción de la imagen o secuencia de planos/escenas si es video,
pensado para guiar a quien diseña/filma, se use IA o no. Se guarda
como sugerenciaVisual, entra en el diff de reimportación, y se agregó
la columna a la plantilla Excel con su explicación en Instrucciones.
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
+++ b/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:A47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -667,100 +667,107 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>• Sugerencia de pieza creativa: cómo se imagina la pieza visualmente -- descripción de la imagen, o secuencia de escenas/planos si es un video (distinto del prompt de IA de arriba, es para guiar a quien diseña/filma, se use o no IA).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>VALORES VÁLIDOS POR COLUMNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
+          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
+          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
+          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
+          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
+          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
+          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
+          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
-    </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos, asignación a alguien del equipo) se completan después, ya adentro del hub.</t>
         </is>
@@ -777,7 +784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -794,7 +801,7 @@
     <col width="40" customWidth="1" min="12" max="12"/>
     <col width="40" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
     <col width="24" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
@@ -873,25 +880,30 @@
       </c>
       <c r="O1" s="4" t="inlineStr">
         <is>
+          <t>Sugerencia de pieza creativa</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
           <t>Pauta</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>Link pieza terminada</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>Link material de referencia</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Notas internas</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>Pilar / fase (referencia interna, NO se sube al hub)</t>
         </is>
@@ -968,19 +980,24 @@
           <t>Ej: "Foto de producto sobre fondo claro, estilo minimalista, luz natural, sin texto superpuesto"</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>Ej: Plano 1: producto entero sobre mesa de madera clara. Plano 2: primer plano de la mano abriendo el envase. Plano 3: producto servido, luz cálida.</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>Solo orgánico</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr">
         <is>
           <t>Ejemplo de fila — borrala y cargá tus propios contenidos.</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr">
+      <c r="T2" s="5" t="inlineStr">
         <is>
           <t>Septiembre · Ejemplo</t>
         </is>

</xml_diff>